<commit_message>
fix import data intern
</commit_message>
<xml_diff>
--- a/public/StaffData/staff (5).xlsx
+++ b/public/StaffData/staff (5).xlsx
@@ -183,7 +183,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -218,7 +218,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -427,10 +427,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -468,7 +468,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>23</v>
       </c>
@@ -504,6 +504,9 @@
       </c>
       <c r="L2" t="s">
         <v>14</v>
+      </c>
+      <c r="M2">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>